<commit_message>
remove paid transport from workbook contract
</commit_message>
<xml_diff>
--- a/input/gastos_scdp_template.xlsx
+++ b/input/gastos_scdp_template.xlsx
@@ -20,11 +20,10 @@
     <definedName name="ApoioE">OFFSET('APOIO'!$E$1,1,0,MAX(1,'RESUMO GASTOS'!$R$1),1)</definedName>
     <definedName name="ApoioF">OFFSET('APOIO'!$F$1,1,0,MAX(1,'RESUMO GASTOS'!$R$1),1)</definedName>
     <definedName name="ApoioG">OFFSET('APOIO'!$G$1,1,0,MAX(1,'RESUMO GASTOS'!$R$1),1)</definedName>
-    <definedName name="ApoioH">OFFSET('APOIO'!$H$1,1,0,MAX(1,'RESUMO GASTOS'!$R$1),1)</definedName>
-    <definedName name="ApoioJ">OFFSET('APOIO'!$I$1,1,0,MAX(1,'RESUMO GASTOS'!$R$1),1)</definedName>
-    <definedName name="ApoioK">OFFSET('APOIO'!$J$1,1,0,MAX(1,'RESUMO GASTOS'!$R$1),1)</definedName>
-    <definedName name="ApoioL">OFFSET('APOIO'!$K$1,1,0,MAX(1,'RESUMO GASTOS'!$R$1),1)</definedName>
-    <definedName name="ApoioM">OFFSET('APOIO'!$L$1,1,0,MAX(1,'RESUMO GASTOS'!$R$1),1)</definedName>
+    <definedName name="ApoioJ">OFFSET('APOIO'!$H$1,1,0,MAX(1,'RESUMO GASTOS'!$R$1),1)</definedName>
+    <definedName name="ApoioK">OFFSET('APOIO'!$I$1,1,0,MAX(1,'RESUMO GASTOS'!$R$1),1)</definedName>
+    <definedName name="ApoioL">OFFSET('APOIO'!$J$1,1,0,MAX(1,'RESUMO GASTOS'!$R$1),1)</definedName>
+    <definedName name="ApoioM">OFFSET('APOIO'!$K$1,1,0,MAX(1,'RESUMO GASTOS'!$R$1),1)</definedName>
     <definedName name="CodigosDebito">OFFSET('APOIO'!$A$1,1,0,MAX(1,'RESUMO GASTOS'!$R$1),1)</definedName>
     <definedName name="ResumoB">OFFSET('RESUMO GASTOS'!$B$1,1,0,MAX(1,'RESUMO GASTOS'!$R$3),1)</definedName>
     <definedName name="ResumoC">OFFSET('RESUMO GASTOS'!$C$1,1,0,MAX(1,'RESUMO GASTOS'!$R$3),1)</definedName>
@@ -41,7 +40,7 @@
     <definedName name="ResumoN">OFFSET('RESUMO GASTOS'!$N$1,1,0,MAX(1,'RESUMO GASTOS'!$R$3),1)</definedName>
     <definedName name="ResumoO">OFFSET('RESUMO GASTOS'!$O$1,1,0,MAX(1,'RESUMO GASTOS'!$R$3),1)</definedName>
     <definedName name="ResumoP">OFFSET('RESUMO GASTOS'!$P$1,1,0,MAX(1,'RESUMO GASTOS'!$R$3),1)</definedName>
-    <definedName name="SCDPLayoutVersion" hidden="0" function="0" vbProcedure="0">"9"</definedName>
+    <definedName name="SCDPLayoutVersion" hidden="0" function="0" vbProcedure="0">"10"</definedName>
     <definedName name="ViagensA">OFFSET('BASE VIAGENS'!$A$1,1,0,MAX(1,'RESUMO GASTOS'!$R$2),1)</definedName>
     <definedName name="ViagensB">OFFSET('BASE VIAGENS'!$B$1,1,0,MAX(1,'RESUMO GASTOS'!$R$2),1)</definedName>
     <definedName name="ViagensC">OFFSET('BASE VIAGENS'!$C$1,1,0,MAX(1,'RESUMO GASTOS'!$R$2),1)</definedName>
@@ -903,9 +902,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblApoioDebito" displayName="tblApoioDebito" ref="A1:L38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:L38"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblApoioDebito" displayName="tblApoioDebito" ref="A1:K38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:K38"/>
+  <tableColumns count="11">
     <tableColumn id="1" name="Código de débito"/>
     <tableColumn id="2" name="Nome por extenso"/>
     <tableColumn id="3" name="Segmento"/>
@@ -913,11 +912,10 @@
     <tableColumn id="5" name="Transportes distribuído (R$)"/>
     <tableColumn id="6" name="Recurso total (R$)"/>
     <tableColumn id="7" name="Transportes agendado (R$)"/>
-    <tableColumn id="8" name="Transportes pago (R$)"/>
-    <tableColumn id="9" name="Rateio para PPGE (%)"/>
-    <tableColumn id="10" name="Rateio para PPGEL (%)"/>
-    <tableColumn id="11" name="Rateio para PPGH (%)"/>
-    <tableColumn id="12" name="Total utilizado por categoria (R$)"/>
+    <tableColumn id="8" name="Rateio para PPGE (%)"/>
+    <tableColumn id="9" name="Rateio para PPGEL (%)"/>
+    <tableColumn id="10" name="Rateio para PPGH (%)"/>
+    <tableColumn id="11" name="Total utilizado por categoria (R$)"/>
   </tableColumns>
 </table>
 </file>
@@ -3469,7 +3467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="32" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="60" min="1" max="1"/>
@@ -3478,12 +3476,11 @@
     <col width="16" customWidth="1" style="60" min="4" max="4"/>
     <col width="16" customWidth="1" style="60" min="5" max="5"/>
     <col width="16" customWidth="1" style="60" min="6" max="6"/>
-    <col width="14" customWidth="1" style="60" min="7" max="8"/>
-    <col width="14" customWidth="1" style="60" min="8" max="8"/>
+    <col width="14" customWidth="1" style="60" min="7" max="7"/>
+    <col width="12" customWidth="1" style="60" min="8" max="8"/>
     <col width="12" customWidth="1" style="60" min="9" max="9"/>
     <col width="12" customWidth="1" style="60" min="10" max="10"/>
-    <col width="12" customWidth="1" style="60" min="11" max="11"/>
-    <col width="18" customWidth="1" style="60" min="12" max="12"/>
+    <col width="18" customWidth="1" style="60" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="64" customHeight="1" s="61">
@@ -3524,25 +3521,20 @@
       </c>
       <c r="H1" s="123" t="inlineStr">
         <is>
-          <t>Transportes pago (R$)</t>
+          <t>Rateio para PPGE (%)</t>
         </is>
       </c>
       <c r="I1" s="123" t="inlineStr">
         <is>
-          <t>Rateio para PPGE (%)</t>
+          <t>Rateio para PPGEL (%)</t>
         </is>
       </c>
       <c r="J1" s="123" t="inlineStr">
         <is>
-          <t>Rateio para PPGEL (%)</t>
+          <t>Rateio para PPGH (%)</t>
         </is>
       </c>
       <c r="K1" s="123" t="inlineStr">
-        <is>
-          <t>Rateio para PPGH (%)</t>
-        </is>
-      </c>
-      <c r="L1" s="123" t="inlineStr">
         <is>
           <t>Total utilizado por categoria (R$)</t>
         </is>
@@ -3577,13 +3569,10 @@
       <c r="G2" s="64" t="n">
         <v>8974.68</v>
       </c>
-      <c r="H2" s="64" t="n">
-        <v>8114.4</v>
-      </c>
+      <c r="H2" s="60" t="n"/>
       <c r="I2" s="60" t="n"/>
       <c r="J2" s="60" t="n"/>
-      <c r="K2" s="60" t="n"/>
-      <c r="L2" s="64">
+      <c r="K2" s="64">
         <f>IF(A2="","",IF(COUNTIFS(ViagensM,A2,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A2,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A2,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -3617,13 +3606,10 @@
       <c r="G3" s="64" t="n">
         <v>14518.23</v>
       </c>
-      <c r="H3" s="64" t="n">
-        <v>13734</v>
-      </c>
+      <c r="H3" s="60" t="n"/>
       <c r="I3" s="60" t="n"/>
       <c r="J3" s="60" t="n"/>
-      <c r="K3" s="60" t="n"/>
-      <c r="L3" s="64">
+      <c r="K3" s="64">
         <f>IF(A3="","",IF(COUNTIFS(ViagensM,A3,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A3,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A3,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -3657,13 +3643,10 @@
       <c r="G4" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="H4" s="60" t="n"/>
       <c r="I4" s="60" t="n"/>
       <c r="J4" s="60" t="n"/>
-      <c r="K4" s="60" t="n"/>
-      <c r="L4" s="64">
+      <c r="K4" s="64">
         <f>IF(A4="","",IF(COUNTIFS(ViagensM,A4,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A4,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A4,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -3697,13 +3680,10 @@
       <c r="G5" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="H5" s="60" t="n"/>
       <c r="I5" s="60" t="n"/>
       <c r="J5" s="60" t="n"/>
-      <c r="K5" s="60" t="n"/>
-      <c r="L5" s="64">
+      <c r="K5" s="64">
         <f>IF(A5="","",IF(COUNTIFS(ViagensM,A5,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A5,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A5,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -3737,13 +3717,10 @@
       <c r="G6" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="H6" s="60" t="n"/>
       <c r="I6" s="60" t="n"/>
       <c r="J6" s="60" t="n"/>
-      <c r="K6" s="60" t="n"/>
-      <c r="L6" s="64">
+      <c r="K6" s="64">
         <f>IF(A6="","",IF(COUNTIFS(ViagensM,A6,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A6,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A6,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -3777,13 +3754,10 @@
       <c r="G7" s="64" t="n">
         <v>846.96</v>
       </c>
-      <c r="H7" s="64" t="n">
-        <v>195.3</v>
-      </c>
+      <c r="H7" s="60" t="n"/>
       <c r="I7" s="60" t="n"/>
       <c r="J7" s="60" t="n"/>
-      <c r="K7" s="60" t="n"/>
-      <c r="L7" s="64">
+      <c r="K7" s="64">
         <f>IF(A7="","",IF(COUNTIFS(ViagensM,A7,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A7,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A7,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -3817,13 +3791,10 @@
       <c r="G8" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="H8" s="60" t="n"/>
       <c r="I8" s="60" t="n"/>
       <c r="J8" s="60" t="n"/>
-      <c r="K8" s="60" t="n"/>
-      <c r="L8" s="64">
+      <c r="K8" s="64">
         <f>IF(A8="","",IF(COUNTIFS(ViagensM,A8,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A8,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A8,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -3857,13 +3828,10 @@
       <c r="G9" s="64" t="n">
         <v>506.1</v>
       </c>
-      <c r="H9" s="64" t="n">
-        <v>506.1</v>
-      </c>
+      <c r="H9" s="60" t="n"/>
       <c r="I9" s="60" t="n"/>
       <c r="J9" s="60" t="n"/>
-      <c r="K9" s="60" t="n"/>
-      <c r="L9" s="64">
+      <c r="K9" s="64">
         <f>IF(A9="","",IF(COUNTIFS(ViagensM,A9,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A9,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A9,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -3897,13 +3865,10 @@
       <c r="G10" s="64" t="n">
         <v>134.44</v>
       </c>
-      <c r="H10" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="H10" s="60" t="n"/>
       <c r="I10" s="60" t="n"/>
       <c r="J10" s="60" t="n"/>
-      <c r="K10" s="60" t="n"/>
-      <c r="L10" s="64">
+      <c r="K10" s="64">
         <f>IF(A10="","",IF(COUNTIFS(ViagensM,A10,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A10,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A10,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -3937,13 +3902,10 @@
       <c r="G11" s="64" t="n">
         <v>9427.92</v>
       </c>
-      <c r="H11" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="H11" s="60" t="n"/>
       <c r="I11" s="60" t="n"/>
       <c r="J11" s="60" t="n"/>
-      <c r="K11" s="60" t="n"/>
-      <c r="L11" s="64">
+      <c r="K11" s="64">
         <f>IF(A11="","",IF(COUNTIFS(ViagensM,A11,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A11,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A11,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -3977,13 +3939,10 @@
       <c r="G12" s="64" t="n">
         <v>9689.1</v>
       </c>
-      <c r="H12" s="64" t="n">
-        <v>862.8</v>
-      </c>
+      <c r="H12" s="60" t="n"/>
       <c r="I12" s="60" t="n"/>
       <c r="J12" s="60" t="n"/>
-      <c r="K12" s="60" t="n"/>
-      <c r="L12" s="64">
+      <c r="K12" s="64">
         <f>IF(A12="","",IF(COUNTIFS(ViagensM,A12,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A12,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A12,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4017,13 +3976,10 @@
       <c r="G13" s="64" t="n">
         <v>1279.52</v>
       </c>
-      <c r="H13" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="H13" s="60" t="n"/>
       <c r="I13" s="60" t="n"/>
       <c r="J13" s="60" t="n"/>
-      <c r="K13" s="60" t="n"/>
-      <c r="L13" s="64">
+      <c r="K13" s="64">
         <f>IF(A13="","",IF(COUNTIFS(ViagensM,A13,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A13,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A13,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4057,13 +4013,10 @@
       <c r="G14" s="64" t="n">
         <v>7074.72</v>
       </c>
-      <c r="H14" s="64" t="n">
-        <v>7074.72</v>
-      </c>
+      <c r="H14" s="60" t="n"/>
       <c r="I14" s="60" t="n"/>
       <c r="J14" s="60" t="n"/>
-      <c r="K14" s="60" t="n"/>
-      <c r="L14" s="64">
+      <c r="K14" s="64">
         <f>IF(A14="","",IF(COUNTIFS(ViagensM,A14,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A14,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A14,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4097,13 +4050,10 @@
       <c r="G15" s="64" t="n">
         <v>1759.22</v>
       </c>
-      <c r="H15" s="64" t="n">
-        <v>1042.14</v>
-      </c>
+      <c r="H15" s="60" t="n"/>
       <c r="I15" s="60" t="n"/>
       <c r="J15" s="60" t="n"/>
-      <c r="K15" s="60" t="n"/>
-      <c r="L15" s="64">
+      <c r="K15" s="64">
         <f>IF(A15="","",IF(COUNTIFS(ViagensM,A15,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A15,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A15,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4137,13 +4087,10 @@
       <c r="G16" s="64" t="n">
         <v>2380.56</v>
       </c>
-      <c r="H16" s="64" t="n">
-        <v>235.2</v>
-      </c>
+      <c r="H16" s="60" t="n"/>
       <c r="I16" s="60" t="n"/>
       <c r="J16" s="60" t="n"/>
-      <c r="K16" s="60" t="n"/>
-      <c r="L16" s="64">
+      <c r="K16" s="64">
         <f>IF(A16="","",IF(COUNTIFS(ViagensM,A16,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A16,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A16,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4177,13 +4124,10 @@
       <c r="G17" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="H17" s="60" t="n"/>
       <c r="I17" s="60" t="n"/>
       <c r="J17" s="60" t="n"/>
-      <c r="K17" s="60" t="n"/>
-      <c r="L17" s="64">
+      <c r="K17" s="64">
         <f>IF(A17="","",IF(COUNTIFS(ViagensM,A17,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A17,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A17,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4217,13 +4161,10 @@
       <c r="G18" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="H18" s="60" t="n"/>
       <c r="I18" s="60" t="n"/>
       <c r="J18" s="60" t="n"/>
-      <c r="K18" s="60" t="n"/>
-      <c r="L18" s="64">
+      <c r="K18" s="64">
         <f>IF(A18="","",IF(COUNTIFS(ViagensM,A18,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A18,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A18,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4257,13 +4198,10 @@
       <c r="G19" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="H19" s="60" t="n"/>
       <c r="I19" s="60" t="n"/>
       <c r="J19" s="60" t="n"/>
-      <c r="K19" s="60" t="n"/>
-      <c r="L19" s="64">
+      <c r="K19" s="64">
         <f>IF(A19="","",IF(COUNTIFS(ViagensM,A19,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A19,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A19,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4297,13 +4235,10 @@
       <c r="G20" s="64" t="n">
         <v>6955.2</v>
       </c>
-      <c r="H20" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="H20" s="60" t="n"/>
       <c r="I20" s="60" t="n"/>
       <c r="J20" s="60" t="n"/>
-      <c r="K20" s="60" t="n"/>
-      <c r="L20" s="64">
+      <c r="K20" s="64">
         <f>IF(A20="","",IF(COUNTIFS(ViagensM,A20,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A20,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A20,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4331,17 +4266,16 @@
         <v/>
       </c>
       <c r="G21" s="64" t="n"/>
-      <c r="H21" s="64" t="n"/>
+      <c r="H21" s="66" t="n">
+        <v>0.333333333333333</v>
+      </c>
       <c r="I21" s="66" t="n">
         <v>0.333333333333333</v>
       </c>
       <c r="J21" s="66" t="n">
         <v>0.333333333333333</v>
       </c>
-      <c r="K21" s="66" t="n">
-        <v>0.333333333333333</v>
-      </c>
-      <c r="L21" s="64">
+      <c r="K21" s="64">
         <f>IF(A21="","",IF(COUNTIFS(ViagensM,A21,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A21,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A21,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4375,13 +4309,10 @@
       <c r="G22" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="H22" s="60" t="n"/>
       <c r="I22" s="60" t="n"/>
       <c r="J22" s="60" t="n"/>
-      <c r="K22" s="60" t="n"/>
-      <c r="L22" s="64">
+      <c r="K22" s="64">
         <f>IF(A22="","",IF(COUNTIFS(ViagensM,A22,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A22,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A22,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4415,13 +4346,10 @@
       <c r="G23" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="H23" s="60" t="n"/>
       <c r="I23" s="60" t="n"/>
       <c r="J23" s="60" t="n"/>
-      <c r="K23" s="60" t="n"/>
-      <c r="L23" s="64">
+      <c r="K23" s="64">
         <f>IF(A23="","",IF(COUNTIFS(ViagensM,A23,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A23,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A23,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4455,13 +4383,10 @@
       <c r="G24" s="64" t="n">
         <v>534.08</v>
       </c>
-      <c r="H24" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="H24" s="60" t="n"/>
       <c r="I24" s="60" t="n"/>
       <c r="J24" s="60" t="n"/>
-      <c r="K24" s="60" t="n"/>
-      <c r="L24" s="64">
+      <c r="K24" s="64">
         <f>IF(A24="","",IF(COUNTIFS(ViagensM,A24,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A24,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A24,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4495,13 +4420,10 @@
       <c r="G25" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="H25" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="H25" s="60" t="n"/>
       <c r="I25" s="60" t="n"/>
       <c r="J25" s="60" t="n"/>
-      <c r="K25" s="60" t="n"/>
-      <c r="L25" s="64">
+      <c r="K25" s="64">
         <f>IF(A25="","",IF(COUNTIFS(ViagensM,A25,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A25,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A25,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4535,13 +4457,10 @@
       <c r="G26" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="H26" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="H26" s="60" t="n"/>
       <c r="I26" s="60" t="n"/>
       <c r="J26" s="60" t="n"/>
-      <c r="K26" s="60" t="n"/>
-      <c r="L26" s="64">
+      <c r="K26" s="64">
         <f>IF(A26="","",IF(COUNTIFS(ViagensM,A26,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A26,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A26,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4575,13 +4494,10 @@
       <c r="G27" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="H27" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="H27" s="60" t="n"/>
       <c r="I27" s="60" t="n"/>
       <c r="J27" s="60" t="n"/>
-      <c r="K27" s="60" t="n"/>
-      <c r="L27" s="64">
+      <c r="K27" s="64">
         <f>IF(A27="","",IF(COUNTIFS(ViagensM,A27,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A27,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A27,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4615,13 +4531,10 @@
       <c r="G28" s="64" t="n">
         <v>1142.1</v>
       </c>
-      <c r="H28" s="64" t="n">
-        <v>453.6</v>
-      </c>
+      <c r="H28" s="60" t="n"/>
       <c r="I28" s="60" t="n"/>
       <c r="J28" s="60" t="n"/>
-      <c r="K28" s="60" t="n"/>
-      <c r="L28" s="64">
+      <c r="K28" s="64">
         <f>IF(A28="","",IF(COUNTIFS(ViagensM,A28,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A28,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A28,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4649,11 +4562,10 @@
         <v/>
       </c>
       <c r="G29" s="64" t="n"/>
-      <c r="H29" s="64" t="n"/>
+      <c r="H29" s="60" t="n"/>
       <c r="I29" s="60" t="n"/>
       <c r="J29" s="60" t="n"/>
-      <c r="K29" s="60" t="n"/>
-      <c r="L29" s="64">
+      <c r="K29" s="64">
         <f>IF(A29="","",IF(COUNTIFS(ViagensM,A29,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A29,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A29,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4681,11 +4593,10 @@
         <v/>
       </c>
       <c r="G30" s="64" t="n"/>
-      <c r="H30" s="64" t="n"/>
+      <c r="H30" s="60" t="n"/>
       <c r="I30" s="60" t="n"/>
       <c r="J30" s="60" t="n"/>
-      <c r="K30" s="60" t="n"/>
-      <c r="L30" s="64">
+      <c r="K30" s="64">
         <f>IF(A30="","",IF(COUNTIFS(ViagensM,A30,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A30,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A30,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4713,11 +4624,10 @@
         <v/>
       </c>
       <c r="G31" s="64" t="n"/>
-      <c r="H31" s="64" t="n"/>
+      <c r="H31" s="60" t="n"/>
       <c r="I31" s="60" t="n"/>
       <c r="J31" s="60" t="n"/>
-      <c r="K31" s="60" t="n"/>
-      <c r="L31" s="64">
+      <c r="K31" s="64">
         <f>IF(A31="","",IF(COUNTIFS(ViagensM,A31,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A31,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A31,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4745,11 +4655,10 @@
         <v/>
       </c>
       <c r="G32" s="64" t="n"/>
-      <c r="H32" s="64" t="n"/>
+      <c r="H32" s="60" t="n"/>
       <c r="I32" s="60" t="n"/>
       <c r="J32" s="60" t="n"/>
-      <c r="K32" s="60" t="n"/>
-      <c r="L32" s="64">
+      <c r="K32" s="64">
         <f>IF(A32="","",IF(COUNTIFS(ViagensM,A32,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A32,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A32,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4777,11 +4686,10 @@
         <v/>
       </c>
       <c r="G33" s="64" t="n"/>
-      <c r="H33" s="64" t="n"/>
+      <c r="H33" s="60" t="n"/>
       <c r="I33" s="60" t="n"/>
       <c r="J33" s="60" t="n"/>
-      <c r="K33" s="60" t="n"/>
-      <c r="L33" s="64">
+      <c r="K33" s="64">
         <f>IF(A33="","",IF(COUNTIFS(ViagensM,A33,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A33,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A33,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4809,11 +4717,10 @@
         <v/>
       </c>
       <c r="G34" s="64" t="n"/>
-      <c r="H34" s="64" t="n"/>
+      <c r="H34" s="60" t="n"/>
       <c r="I34" s="60" t="n"/>
       <c r="J34" s="60" t="n"/>
-      <c r="K34" s="60" t="n"/>
-      <c r="L34" s="64">
+      <c r="K34" s="64">
         <f>IF(A34="","",IF(COUNTIFS(ViagensM,A34,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A34,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A34,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4841,11 +4748,10 @@
         <v/>
       </c>
       <c r="G35" s="64" t="n"/>
-      <c r="H35" s="64" t="n"/>
+      <c r="H35" s="60" t="n"/>
       <c r="I35" s="60" t="n"/>
       <c r="J35" s="60" t="n"/>
-      <c r="K35" s="60" t="n"/>
-      <c r="L35" s="64">
+      <c r="K35" s="64">
         <f>IF(A35="","",IF(COUNTIFS(ViagensM,A35,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A35,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A35,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4879,13 +4785,10 @@
       <c r="G36" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="H36" s="60" t="n"/>
       <c r="I36" s="60" t="n"/>
       <c r="J36" s="60" t="n"/>
-      <c r="K36" s="60" t="n"/>
-      <c r="L36" s="64">
+      <c r="K36" s="64">
         <f>IF(A36="","",IF(COUNTIFS(ViagensM,A36,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A36,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A36,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>
@@ -4913,11 +4816,10 @@
         <v/>
       </c>
       <c r="G37" s="64" t="n"/>
-      <c r="H37" s="64" t="n"/>
+      <c r="H37" s="60" t="n"/>
       <c r="I37" s="60" t="n"/>
       <c r="J37" s="60" t="n"/>
-      <c r="K37" s="60" t="n"/>
-      <c r="L37" s="64">
+      <c r="K37" s="64">
         <f>IF(A37="","",IF(COUNTIFS(ViagensM,A37,ViagensC,"Cancelada",ViagensN,"")&gt;0,"Pendente",SUMIFS(ViagensK,ViagensM,A37,ViagensC,"&lt;&gt;Cancelada")+SUMIFS(ViagensK,ViagensM,A37,ViagensC,"Cancelada",ViagensN,"Sim")))</f>
         <v/>
       </c>

</xml_diff>